<commit_message>
Actualizacion del esquematico , adicion de los datasheet a las documentacion e inicio de la PCB
</commit_message>
<xml_diff>
--- a/Documentacion/Presupuesto.xlsx
+++ b/Documentacion/Presupuesto.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesro\Desktop\Sumo Robot\Sumo_Bot_El_Empujon\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81A5F90C-2C81-4F46-9085-FCAFEB4EB969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF82D88B-120E-47FE-8E6D-88194B79C4BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D2BAF053-7DE6-4243-82FB-AD2ADD9EC4EA}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>Microcontrolador</t>
   </si>
   <si>
-    <t>JGB37-520 (12V, 300-400 RPM, caja metálica)</t>
-  </si>
-  <si>
     <t>Driver de Potencia</t>
   </si>
   <si>
@@ -165,6 +162,9 @@
   </si>
   <si>
     <t>Precio unitario en DOP</t>
+  </si>
+  <si>
+    <t>JGA25-371</t>
   </si>
 </sst>
 </file>
@@ -316,37 +316,6 @@
   <dxfs count="10">
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <name val="Times New Roman"/>
-        <family val="1"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -386,6 +355,25 @@
         <family val="1"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -524,6 +512,18 @@
         </left>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -538,19 +538,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{56FB128F-CE2D-4622-840D-F8F6809678F4}" name="Table1" displayName="Table1" ref="C3:J15" totalsRowShown="0" dataDxfId="1" tableBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{56FB128F-CE2D-4622-840D-F8F6809678F4}" name="Table1" displayName="Table1" ref="C3:J15" totalsRowShown="0" dataDxfId="9" tableBorderDxfId="8">
   <autoFilter ref="C3:J15" xr:uid="{56FB128F-CE2D-4622-840D-F8F6809678F4}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C63E0612-C8CC-4D05-9124-D6FE424DE1D0}" name="Componente" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{37C31126-C1C0-453E-B849-2A66DE446D72}" name="Descripción / Modelo Recomendado" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{53C17134-B8D4-4A3F-AB34-ECA1CE877BFF}" name="Cantidad" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{285CBBF9-AA1D-4917-BCD7-E44601C4F76D}" name="Precio en USD" dataDxfId="5" dataCellStyle="Currency"/>
-    <tableColumn id="5" xr3:uid="{7C623A9C-EF69-4319-B211-C3268A231131}" name="Precio en DOP" dataDxfId="4" dataCellStyle="Currency"/>
-    <tableColumn id="8" xr3:uid="{F889BF4B-8588-432D-A4CE-857F512F75A2}" name="Precio unitario en DOP" dataDxfId="0" dataCellStyle="Currency">
+    <tableColumn id="1" xr3:uid="{C63E0612-C8CC-4D05-9124-D6FE424DE1D0}" name="Componente" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{37C31126-C1C0-453E-B849-2A66DE446D72}" name="Descripción / Modelo Recomendado" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{53C17134-B8D4-4A3F-AB34-ECA1CE877BFF}" name="Cantidad" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{285CBBF9-AA1D-4917-BCD7-E44601C4F76D}" name="Precio en USD" dataDxfId="4" dataCellStyle="Currency"/>
+    <tableColumn id="5" xr3:uid="{7C623A9C-EF69-4319-B211-C3268A231131}" name="Precio en DOP" dataDxfId="3" dataCellStyle="Currency"/>
+    <tableColumn id="8" xr3:uid="{F889BF4B-8588-432D-A4CE-857F512F75A2}" name="Precio unitario en DOP" dataDxfId="2" dataCellStyle="Currency">
       <calculatedColumnFormula>Table1[[#This Row],[Precio en DOP]]/Table1[[#This Row],[Cantidad]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{3C4D9860-0BCC-454A-BAA4-AEE4499DBB83}" name="Precio de libra" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{198E9086-D390-40E4-AE15-3C55E9B5FE02}" name="Link de compra" dataDxfId="2" dataCellStyle="Hyperlink"/>
+    <tableColumn id="6" xr3:uid="{3C4D9860-0BCC-454A-BAA4-AEE4499DBB83}" name="Precio de libra" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{198E9086-D390-40E4-AE15-3C55E9B5FE02}" name="Link de compra" dataDxfId="0" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -887,7 +887,7 @@
   <sheetData>
     <row r="2" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="F2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G2">
         <v>61.09</v>
@@ -910,7 +910,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I3" t="s">
         <v>2</v>
@@ -924,7 +924,7 @@
         <v>7</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E4" s="5">
         <v>2</v>
@@ -942,15 +942,15 @@
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="3:10" ht="36.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C5" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
       <c r="E5" s="5">
         <v>2</v>
@@ -968,15 +968,15 @@
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="3:10" ht="18.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C6" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E6" s="5">
         <v>2</v>
@@ -994,15 +994,15 @@
       </c>
       <c r="I6" s="8"/>
       <c r="J6" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="3:10" ht="36.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C7" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E7" s="4">
         <v>3</v>
@@ -1020,15 +1020,15 @@
       </c>
       <c r="I7" s="8"/>
       <c r="J7" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="3:10" ht="18.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C8" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E8" s="4">
         <v>5</v>
@@ -1046,15 +1046,15 @@
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="3:10" ht="36.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C9" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9" s="5">
         <v>2</v>
@@ -1072,15 +1072,15 @@
       </c>
       <c r="I9" s="8"/>
       <c r="J9" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="3:10" ht="36" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>16</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>17</v>
       </c>
       <c r="E10" s="5">
         <v>120</v>
@@ -1098,15 +1098,15 @@
       </c>
       <c r="I10" s="8"/>
       <c r="J10" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="3:10" ht="36" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>25</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>26</v>
       </c>
       <c r="E11" s="5">
         <v>1</v>
@@ -1124,15 +1124,15 @@
       </c>
       <c r="I11" s="8"/>
       <c r="J11" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="3:10" ht="18.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C12" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E12" s="5">
         <v>3</v>
@@ -1150,10 +1150,10 @@
     </row>
     <row r="13" spans="3:10" ht="18.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C13" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E13" s="4">
         <v>1</v>
@@ -1168,15 +1168,15 @@
       </c>
       <c r="I13" s="8"/>
       <c r="J13" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="3:10" ht="18.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="E14" s="4">
         <v>1</v>
@@ -1194,12 +1194,12 @@
       </c>
       <c r="I14" s="8"/>
       <c r="J14" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="3:10" ht="18.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="C15" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>

</xml_diff>

<commit_message>
Generacion del STEP, finalizacion del esquematico y de la PCB, generacion de los archivos de manufactura de la PCB, Pedido de la PCB y actualizacion del Presupuesto.
</commit_message>
<xml_diff>
--- a/Documentacion/Presupuesto.xlsx
+++ b/Documentacion/Presupuesto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wesro\Desktop\Sumo Robot\Sumo_Bot_El_Empujon\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF82D88B-120E-47FE-8E6D-88194B79C4BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4646F21-40C5-4B1D-81F1-1CC1F676591A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D2BAF053-7DE6-4243-82FB-AD2ADD9EC4EA}"/>
   </bookViews>
@@ -1182,15 +1182,15 @@
         <v>1</v>
       </c>
       <c r="F14" s="6">
-        <v>14</v>
+        <v>5.67</v>
       </c>
       <c r="G14" s="11">
         <f>$G$2*F14</f>
-        <v>855.26</v>
+        <v>346.38030000000003</v>
       </c>
       <c r="H14" s="11">
         <f>Table1[[#This Row],[Precio en DOP]]/Table1[[#This Row],[Cantidad]]</f>
-        <v>855.26</v>
+        <v>346.38030000000003</v>
       </c>
       <c r="I14" s="8"/>
       <c r="J14" s="9" t="s">
@@ -1206,7 +1206,7 @@
       <c r="F15" s="13"/>
       <c r="G15" s="7">
         <f>SUM(G4:G14)</f>
-        <v>6459.9452000000001</v>
+        <v>5951.0654999999997</v>
       </c>
       <c r="H15" s="7"/>
       <c r="I15" s="8"/>

</xml_diff>